<commit_message>
Backup 18.08.25 (vor paintings by)
</commit_message>
<xml_diff>
--- a/Monitoring/TimeMonitoring.xlsx
+++ b/Monitoring/TimeMonitoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tim/NoteDeck/Monitoring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A72F71-22FC-984E-8D27-861F2AA87A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{352706A0-0DD5-8D48-8B44-792A00536F1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -819,13 +819,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="3" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -857,7 +857,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -873,6 +873,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4512,7 +4513,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB66FF37-F629-234C-BA15-F7C53EAAE600}">
-  <dimension ref="C6:P159"/>
+  <dimension ref="C6:P160"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="17" width="17.83203125" customWidth="1"/>
@@ -4607,13 +4608,13 @@
       <c r="E8" t="s">
         <v>213</v>
       </c>
-      <c r="F8" s="8"/>
+      <c r="F8" s="10"/>
       <c r="K8" s="9"/>
       <c r="L8" s="9"/>
       <c r="M8" s="9"/>
       <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
     </row>
     <row r="9" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E9" t="s">
@@ -4623,8 +4624,8 @@
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
       <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
     </row>
     <row r="10" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E10" t="s">
@@ -4634,8 +4635,8 @@
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
       <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
     </row>
     <row r="11" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E11" t="s">
@@ -4645,8 +4646,8 @@
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
       <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
     </row>
     <row r="12" spans="3:16" x14ac:dyDescent="0.2">
       <c r="D12" t="s">
@@ -4655,13 +4656,13 @@
       <c r="E12" t="s">
         <v>213</v>
       </c>
-      <c r="F12" s="8"/>
+      <c r="F12" s="10"/>
       <c r="K12" s="9"/>
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>
       <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
     </row>
     <row r="13" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E13" t="s">
@@ -4671,8 +4672,8 @@
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
       <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
     </row>
     <row r="14" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E14" t="s">
@@ -4682,8 +4683,8 @@
       <c r="L14" s="9"/>
       <c r="M14" s="9"/>
       <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
     </row>
     <row r="15" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E15" t="s">
@@ -4693,8 +4694,8 @@
       <c r="L15" s="9"/>
       <c r="M15" s="9"/>
       <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
     </row>
     <row r="16" spans="3:16" x14ac:dyDescent="0.2">
       <c r="D16" t="s">
@@ -4703,13 +4704,13 @@
       <c r="E16" t="s">
         <v>213</v>
       </c>
-      <c r="F16" s="8"/>
+      <c r="F16" s="10"/>
       <c r="K16" s="9"/>
       <c r="L16" s="9"/>
       <c r="M16" s="9"/>
       <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
     </row>
     <row r="17" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E17" t="s">
@@ -4719,20 +4720,20 @@
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
       <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="9"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
     </row>
     <row r="18" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E18" t="s">
         <v>214</v>
       </c>
-      <c r="F18" s="8"/>
+      <c r="F18" s="10"/>
       <c r="K18" s="9"/>
       <c r="L18" s="9"/>
       <c r="M18" s="9"/>
       <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="9"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
     </row>
     <row r="19" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E19" t="s">
@@ -4742,8 +4743,8 @@
       <c r="L19" s="9"/>
       <c r="M19" s="9"/>
       <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="9"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="8"/>
     </row>
     <row r="20" spans="4:16" x14ac:dyDescent="0.2">
       <c r="D20" t="s">
@@ -4752,13 +4753,13 @@
       <c r="E20" t="s">
         <v>213</v>
       </c>
-      <c r="F20" s="8"/>
+      <c r="F20" s="10"/>
       <c r="K20" s="9"/>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="9"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
     </row>
     <row r="21" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E21" t="s">
@@ -4768,20 +4769,20 @@
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="9"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
     </row>
     <row r="22" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E22" t="s">
         <v>214</v>
       </c>
-      <c r="F22" s="8"/>
+      <c r="F22" s="10"/>
       <c r="K22" s="9"/>
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9"/>
-      <c r="O22" s="9"/>
-      <c r="P22" s="9"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
     </row>
     <row r="23" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E23" t="s">
@@ -4791,8 +4792,8 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9"/>
-      <c r="O23" s="9"/>
-      <c r="P23" s="9"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
     </row>
     <row r="24" spans="4:16" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
@@ -4801,13 +4802,13 @@
       <c r="E24" t="s">
         <v>213</v>
       </c>
-      <c r="F24" s="8"/>
+      <c r="F24" s="10"/>
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="9"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
     </row>
     <row r="25" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E25" t="s">
@@ -4817,20 +4818,20 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9"/>
-      <c r="O25" s="9"/>
-      <c r="P25" s="9"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
     </row>
     <row r="26" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E26" t="s">
         <v>214</v>
       </c>
-      <c r="F26" s="8"/>
+      <c r="F26" s="10"/>
       <c r="K26" s="9"/>
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
-      <c r="P26" s="9"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
     </row>
     <row r="27" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E27" t="s">
@@ -4840,8 +4841,8 @@
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9"/>
-      <c r="O27" s="9"/>
-      <c r="P27" s="9"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
     </row>
     <row r="28" spans="4:16" x14ac:dyDescent="0.2">
       <c r="D28" t="s">
@@ -4850,13 +4851,13 @@
       <c r="E28" t="s">
         <v>213</v>
       </c>
-      <c r="F28" s="8"/>
+      <c r="F28" s="10"/>
       <c r="K28" s="9"/>
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="9"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
     </row>
     <row r="29" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E29" t="s">
@@ -4866,19 +4867,20 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9"/>
-      <c r="O29" s="9"/>
-      <c r="P29" s="9"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
     </row>
     <row r="30" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E30" t="s">
         <v>214</v>
       </c>
+      <c r="F30" s="10"/>
       <c r="K30" s="9"/>
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9"/>
-      <c r="O30" s="9"/>
-      <c r="P30" s="9"/>
+      <c r="O30" s="8"/>
+      <c r="P30" s="8"/>
     </row>
     <row r="31" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E31" t="s">
@@ -4888,8 +4890,8 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9"/>
-      <c r="O31" s="9"/>
-      <c r="P31" s="9"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
     </row>
     <row r="32" spans="4:16" x14ac:dyDescent="0.2">
       <c r="D32" t="s">
@@ -4898,13 +4900,13 @@
       <c r="E32" t="s">
         <v>213</v>
       </c>
-      <c r="F32" s="8"/>
+      <c r="F32" s="10"/>
       <c r="K32" s="9"/>
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9"/>
-      <c r="O32" s="9"/>
-      <c r="P32" s="9"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="8"/>
     </row>
     <row r="33" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E33" t="s">
@@ -4914,8 +4916,8 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9"/>
-      <c r="O33" s="9"/>
-      <c r="P33" s="9"/>
+      <c r="O33" s="8"/>
+      <c r="P33" s="8"/>
     </row>
     <row r="34" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E34" t="s">
@@ -4925,8 +4927,8 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="9"/>
+      <c r="O34" s="8"/>
+      <c r="P34" s="8"/>
     </row>
     <row r="35" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E35" t="s">
@@ -4936,8 +4938,8 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="9"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
     </row>
     <row r="36" spans="4:16" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
@@ -4946,13 +4948,13 @@
       <c r="E36" t="s">
         <v>213</v>
       </c>
-      <c r="F36" s="8"/>
+      <c r="F36" s="10"/>
       <c r="K36" s="9"/>
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
-      <c r="P36" s="9"/>
+      <c r="O36" s="8"/>
+      <c r="P36" s="8"/>
     </row>
     <row r="37" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E37" t="s">
@@ -4962,8 +4964,8 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9"/>
-      <c r="O37" s="9"/>
-      <c r="P37" s="9"/>
+      <c r="O37" s="8"/>
+      <c r="P37" s="8"/>
     </row>
     <row r="38" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E38" t="s">
@@ -4973,8 +4975,8 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9"/>
-      <c r="O38" s="9"/>
-      <c r="P38" s="9"/>
+      <c r="O38" s="8"/>
+      <c r="P38" s="8"/>
     </row>
     <row r="39" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E39" t="s">
@@ -4984,8 +4986,8 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9"/>
-      <c r="O39" s="9"/>
-      <c r="P39" s="9"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="8"/>
     </row>
     <row r="40" spans="4:16" x14ac:dyDescent="0.2">
       <c r="D40" t="s">
@@ -4994,13 +4996,13 @@
       <c r="E40" t="s">
         <v>213</v>
       </c>
-      <c r="F40" s="8"/>
+      <c r="F40" s="10"/>
       <c r="K40" s="9"/>
       <c r="L40" s="9"/>
       <c r="M40" s="9"/>
       <c r="N40" s="9"/>
-      <c r="O40" s="9"/>
-      <c r="P40" s="9"/>
+      <c r="O40" s="8"/>
+      <c r="P40" s="8"/>
     </row>
     <row r="41" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E41" t="s">
@@ -5010,8 +5012,8 @@
       <c r="L41" s="9"/>
       <c r="M41" s="9"/>
       <c r="N41" s="9"/>
-      <c r="O41" s="9"/>
-      <c r="P41" s="9"/>
+      <c r="O41" s="8"/>
+      <c r="P41" s="8"/>
     </row>
     <row r="42" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E42" t="s">
@@ -5021,8 +5023,8 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9"/>
-      <c r="O42" s="9"/>
-      <c r="P42" s="9"/>
+      <c r="O42" s="8"/>
+      <c r="P42" s="8"/>
     </row>
     <row r="43" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E43" t="s">
@@ -5032,8 +5034,8 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9"/>
-      <c r="O43" s="9"/>
-      <c r="P43" s="9"/>
+      <c r="O43" s="8"/>
+      <c r="P43" s="8"/>
     </row>
     <row r="44" spans="4:16" x14ac:dyDescent="0.2">
       <c r="D44" t="s">
@@ -5042,13 +5044,13 @@
       <c r="E44" t="s">
         <v>213</v>
       </c>
-      <c r="F44" s="8"/>
+      <c r="F44" s="10"/>
       <c r="K44" s="9"/>
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
-      <c r="O44" s="9"/>
-      <c r="P44" s="9"/>
+      <c r="O44" s="8"/>
+      <c r="P44" s="8"/>
     </row>
     <row r="45" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E45" t="s">
@@ -5058,8 +5060,8 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9"/>
-      <c r="O45" s="9"/>
-      <c r="P45" s="9"/>
+      <c r="O45" s="8"/>
+      <c r="P45" s="8"/>
     </row>
     <row r="46" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E46" t="s">
@@ -5069,8 +5071,8 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9"/>
-      <c r="O46" s="9"/>
-      <c r="P46" s="9"/>
+      <c r="O46" s="8"/>
+      <c r="P46" s="8"/>
     </row>
     <row r="47" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E47" t="s">
@@ -5080,8 +5082,8 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9"/>
-      <c r="O47" s="9"/>
-      <c r="P47" s="9"/>
+      <c r="O47" s="8"/>
+      <c r="P47" s="8"/>
     </row>
     <row r="48" spans="4:16" x14ac:dyDescent="0.2">
       <c r="D48" t="s">
@@ -5090,13 +5092,13 @@
       <c r="E48" t="s">
         <v>213</v>
       </c>
-      <c r="F48" s="8"/>
+      <c r="F48" s="10"/>
       <c r="K48" s="9"/>
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9"/>
-      <c r="O48" s="9"/>
-      <c r="P48" s="9"/>
+      <c r="O48" s="8"/>
+      <c r="P48" s="8"/>
     </row>
     <row r="49" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E49" t="s">
@@ -5106,8 +5108,8 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9"/>
-      <c r="O49" s="9"/>
-      <c r="P49" s="9"/>
+      <c r="O49" s="8"/>
+      <c r="P49" s="8"/>
     </row>
     <row r="50" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E50" t="s">
@@ -5117,8 +5119,8 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9"/>
-      <c r="O50" s="9"/>
-      <c r="P50" s="9"/>
+      <c r="O50" s="8"/>
+      <c r="P50" s="8"/>
     </row>
     <row r="51" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E51" t="s">
@@ -5128,8 +5130,8 @@
       <c r="L51" s="9"/>
       <c r="M51" s="9"/>
       <c r="N51" s="9"/>
-      <c r="O51" s="9"/>
-      <c r="P51" s="9"/>
+      <c r="O51" s="8"/>
+      <c r="P51" s="8"/>
     </row>
     <row r="52" spans="3:16" x14ac:dyDescent="0.2">
       <c r="D52" t="s">
@@ -5138,13 +5140,13 @@
       <c r="E52" t="s">
         <v>213</v>
       </c>
-      <c r="F52" s="8"/>
+      <c r="F52" s="10"/>
       <c r="K52" s="9"/>
       <c r="L52" s="9"/>
       <c r="M52" s="9"/>
       <c r="N52" s="9"/>
-      <c r="O52" s="9"/>
-      <c r="P52" s="9"/>
+      <c r="O52" s="8"/>
+      <c r="P52" s="8"/>
     </row>
     <row r="53" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E53" t="s">
@@ -5154,8 +5156,8 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9"/>
-      <c r="O53" s="9"/>
-      <c r="P53" s="9"/>
+      <c r="O53" s="8"/>
+      <c r="P53" s="8"/>
     </row>
     <row r="54" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E54" t="s">
@@ -5165,8 +5167,8 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9"/>
-      <c r="O54" s="9"/>
-      <c r="P54" s="9"/>
+      <c r="O54" s="8"/>
+      <c r="P54" s="8"/>
     </row>
     <row r="55" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E55" t="s">
@@ -5176,8 +5178,8 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9"/>
-      <c r="O55" s="9"/>
-      <c r="P55" s="9"/>
+      <c r="O55" s="8"/>
+      <c r="P55" s="8"/>
     </row>
     <row r="56" spans="3:16" x14ac:dyDescent="0.2">
       <c r="D56" t="s">
@@ -5186,13 +5188,13 @@
       <c r="E56" t="s">
         <v>213</v>
       </c>
-      <c r="F56" s="8"/>
+      <c r="F56" s="10"/>
       <c r="K56" s="9"/>
       <c r="L56" s="9"/>
       <c r="M56" s="9"/>
       <c r="N56" s="9"/>
-      <c r="O56" s="9"/>
-      <c r="P56" s="9"/>
+      <c r="O56" s="8"/>
+      <c r="P56" s="8"/>
     </row>
     <row r="57" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E57" t="s">
@@ -5202,8 +5204,8 @@
       <c r="L57" s="9"/>
       <c r="M57" s="9"/>
       <c r="N57" s="9"/>
-      <c r="O57" s="9"/>
-      <c r="P57" s="9"/>
+      <c r="O57" s="8"/>
+      <c r="P57" s="8"/>
     </row>
     <row r="58" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E58" t="s">
@@ -5213,8 +5215,8 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9"/>
-      <c r="O58" s="9"/>
-      <c r="P58" s="9"/>
+      <c r="O58" s="8"/>
+      <c r="P58" s="8"/>
     </row>
     <row r="59" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E59" t="s">
@@ -5224,572 +5226,585 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9"/>
-      <c r="O59" s="9"/>
-      <c r="P59" s="9"/>
+      <c r="O59" s="8"/>
+      <c r="P59" s="8"/>
     </row>
     <row r="60" spans="3:16" x14ac:dyDescent="0.2">
-      <c r="C60" t="s">
+      <c r="K60" s="9"/>
+      <c r="L60" s="9"/>
+      <c r="M60" s="9"/>
+      <c r="N60" s="9"/>
+      <c r="O60" s="8"/>
+      <c r="P60" s="8"/>
+    </row>
+    <row r="61" spans="3:16" x14ac:dyDescent="0.2">
+      <c r="C61" t="s">
         <v>53</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D61" t="s">
         <v>217</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E61" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="61" spans="3:16" x14ac:dyDescent="0.2">
-      <c r="E61" t="s">
-        <v>216</v>
-      </c>
+      <c r="K61" s="9"/>
+      <c r="L61" s="9"/>
+      <c r="M61" s="9"/>
+      <c r="N61" s="9"/>
     </row>
     <row r="62" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E62" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="63" spans="3:16" x14ac:dyDescent="0.2">
       <c r="E63" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="64" spans="3:16" x14ac:dyDescent="0.2">
+      <c r="E64" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="64" spans="3:16" x14ac:dyDescent="0.2">
-      <c r="D64" t="s">
+    <row r="65" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D65" t="s">
         <v>218</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E65" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="65" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E65" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="66" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E66" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="67" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E67" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="68" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E68" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="68" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D68" t="s">
+    <row r="69" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D69" t="s">
         <v>219</v>
       </c>
-      <c r="E68" t="s">
+      <c r="E69" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="69" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E69" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="70" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E70" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="71" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E71" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="72" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E72" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="72" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D72" t="s">
+    <row r="73" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D73" t="s">
         <v>220</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E73" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="73" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E73" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="74" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E74" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="75" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E75" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="76" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E76" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="76" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D76" t="s">
+    <row r="77" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D77" t="s">
         <v>221</v>
       </c>
-      <c r="E76" t="s">
+      <c r="E77" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="77" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E77" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="78" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E78" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="79" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E79" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="80" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E80" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="80" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D80" t="s">
+    <row r="81" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D81" t="s">
         <v>222</v>
       </c>
-      <c r="E80" t="s">
+      <c r="E81" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="81" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E81" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="82" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E82" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="83" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E83" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="84" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E84" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="84" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D84" t="s">
+    <row r="85" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D85" t="s">
         <v>223</v>
       </c>
-      <c r="E84" t="s">
+      <c r="E85" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="85" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E85" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="86" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E86" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="87" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E87" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="88" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E88" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="88" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D88" t="s">
+    <row r="89" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D89" t="s">
         <v>224</v>
       </c>
-      <c r="E88" t="s">
+      <c r="E89" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="89" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E89" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="90" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E90" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="91" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E91" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="92" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E92" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="92" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D92" t="s">
+    <row r="93" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D93" t="s">
         <v>225</v>
       </c>
-      <c r="E92" t="s">
+      <c r="E93" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="93" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E93" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="94" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E94" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="95" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E95" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="96" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E96" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="96" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D96" t="s">
+    <row r="97" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D97" t="s">
         <v>226</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E97" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="97" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E97" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="98" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E98" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="99" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E99" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="100" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E100" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="100" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D100" t="s">
+    <row r="101" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D101" t="s">
         <v>227</v>
       </c>
-      <c r="E100" t="s">
+      <c r="E101" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="101" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E101" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="102" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E102" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="103" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E103" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="104" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E104" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="104" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D104" t="s">
+    <row r="105" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D105" t="s">
         <v>228</v>
       </c>
-      <c r="E104" t="s">
+      <c r="E105" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="105" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E105" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="106" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E106" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="107" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E107" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="108" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E108" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="108" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D108" t="s">
+    <row r="109" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D109" t="s">
         <v>229</v>
       </c>
-      <c r="E108" t="s">
+      <c r="E109" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="109" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E109" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="110" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E110" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="111" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E111" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="112" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="E112" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="112" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D112" t="s">
+    <row r="113" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D113" t="s">
         <v>230</v>
       </c>
-      <c r="E112" t="s">
+      <c r="E113" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="113" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="E113" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="114" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E114" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="115" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E115" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="116" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E116" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="116" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D116" t="s">
+    <row r="117" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D117" t="s">
         <v>231</v>
       </c>
-      <c r="E116" t="s">
+      <c r="E117" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="117" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="E117" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="118" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E118" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="119" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E119" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="120" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E120" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="120" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D120" t="s">
+    <row r="121" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D121" t="s">
         <v>232</v>
       </c>
-      <c r="E120" t="s">
+      <c r="E121" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="121" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="E121" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="122" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E122" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="123" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E123" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="124" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E124" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="124" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C124" t="s">
+    <row r="125" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C125" t="s">
         <v>184</v>
       </c>
-      <c r="D124" t="s">
+      <c r="D125" t="s">
         <v>233</v>
       </c>
-      <c r="E124" t="s">
+      <c r="E125" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="125" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="E125" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="126" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E126" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="127" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E127" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="128" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E128" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="128" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D128" t="s">
+    <row r="129" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D129" t="s">
         <v>234</v>
       </c>
-      <c r="E128" t="s">
+      <c r="E129" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="129" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E129" t="s">
+    <row r="130" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E130" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="130" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E130" t="s">
+    <row r="131" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E131" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="131" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E131" t="s">
+    <row r="132" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E132" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="132" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D132" t="s">
+    <row r="133" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D133" t="s">
         <v>235</v>
       </c>
-      <c r="E132" t="s">
+      <c r="E133" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="133" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E133" t="s">
+      <c r="F133" s="10"/>
+    </row>
+    <row r="134" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E134" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="134" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E134" t="s">
+    <row r="135" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E135" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="135" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E135" t="s">
+    <row r="136" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E136" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="136" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="D136" t="s">
+    <row r="137" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D137" t="s">
         <v>236</v>
       </c>
-      <c r="E136" t="s">
+      <c r="E137" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="137" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E137" t="s">
+    <row r="138" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E138" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="138" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E138" t="s">
+    <row r="139" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E139" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="139" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E139" t="s">
+    <row r="140" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E140" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="140" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E140" t="s">
+    <row r="141" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E141" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="141" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E141" t="s">
+    <row r="142" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E142" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="142" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E142" t="s">
+    <row r="143" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E143" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="143" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E143" t="s">
+    <row r="144" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="E144" t="s">
         <v>215</v>
-      </c>
-    </row>
-    <row r="144" spans="4:5" x14ac:dyDescent="0.2">
-      <c r="E144" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="145" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E145" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="146" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E146" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="147" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E147" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="148" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E148" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="149" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E149" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="150" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E150" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="151" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E151" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="152" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E152" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="153" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E153" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="154" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E154" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="155" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E155" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="156" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E156" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="157" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E157" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="158" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E158" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="159" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E159" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="160" spans="5:5" x14ac:dyDescent="0.2">
+      <c r="E160" t="s">
         <v>215</v>
       </c>
     </row>

</xml_diff>